<commit_message>
changed the error plot to show avg_max_error and avg_min_error
</commit_message>
<xml_diff>
--- a/results/error_and_stretch_data_with_cut-off_AND_overlap/64/overlap50/64nodes_diameter38_cutoff3.3333333333333335-repetitions50-overlap50.xlsx
+++ b/results/error_and_stretch_data_with_cut-off_AND_overlap/64/overlap50/64nodes_diameter38_cutoff3.3333333333333335-repetitions50-overlap50.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ksuprod-my.sharepoint.com/personal/sbhatt23_kent_edu/Documents/Desktop/Distributed Directories Under Predictions/results/error_and_stretch_data_with_cut-off_AND_overlap/64/overlap50/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_62E33A1910375E164CC78A0C93F1C69C655336A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{499DDC64-047E-46A7-9908-F2E05C7146A6}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="raw" sheetId="1" r:id="rId1"/>
     <sheet name="summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -62,8 +68,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,13 +132,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -170,7 +184,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -204,6 +218,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -238,9 +253,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -413,11 +429,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G251"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -440,15 +456,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -463,15 +479,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -486,15 +502,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4">
-        <v>0.2105</v>
+        <v>0.21049999999999999</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -509,15 +525,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
       <c r="C5">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -532,15 +548,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
       <c r="C6">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -555,9 +571,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -578,15 +594,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8">
-        <v>0.1316</v>
+        <v>0.13159999999999999</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -601,15 +617,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B9">
         <v>2</v>
       </c>
       <c r="C9">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -624,15 +640,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -647,15 +663,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B11">
         <v>2</v>
       </c>
       <c r="C11">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -670,15 +686,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -693,15 +709,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -716,9 +732,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B14">
         <v>2</v>
@@ -739,15 +755,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -762,15 +778,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -785,15 +801,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -808,15 +824,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -831,15 +847,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B19">
         <v>2</v>
       </c>
       <c r="C19">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -854,15 +870,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -877,15 +893,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B21">
         <v>2</v>
       </c>
       <c r="C21">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -900,15 +916,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B22">
         <v>2</v>
       </c>
       <c r="C22">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -923,15 +939,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B23">
         <v>2</v>
       </c>
       <c r="C23">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -946,15 +962,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -969,15 +985,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -992,15 +1008,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B26">
         <v>2</v>
       </c>
       <c r="C26">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1015,15 +1031,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B27">
         <v>2</v>
       </c>
       <c r="C27">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1038,15 +1054,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1061,15 +1077,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B29">
         <v>2</v>
       </c>
       <c r="C29">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1084,15 +1100,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B30">
         <v>2</v>
       </c>
       <c r="C30">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1107,15 +1123,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
       <c r="C31">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1130,15 +1146,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B32">
         <v>2</v>
       </c>
       <c r="C32">
-        <v>0.2105</v>
+        <v>0.21049999999999999</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1153,15 +1169,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B33">
         <v>2</v>
       </c>
       <c r="C33">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1176,15 +1192,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B34">
         <v>2</v>
       </c>
       <c r="C34">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1199,15 +1215,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B35">
         <v>2</v>
       </c>
       <c r="C35">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -1222,15 +1238,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B36">
         <v>2</v>
       </c>
       <c r="C36">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -1245,15 +1261,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B37">
         <v>2</v>
       </c>
       <c r="C37">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1268,15 +1284,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B38">
         <v>2</v>
       </c>
       <c r="C38">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1291,15 +1307,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B39">
         <v>2</v>
       </c>
       <c r="C39">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1314,15 +1330,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B40">
         <v>2</v>
       </c>
       <c r="C40">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1337,15 +1353,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B41">
         <v>2</v>
       </c>
       <c r="C41">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1360,15 +1376,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B42">
         <v>2</v>
       </c>
       <c r="C42">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1383,9 +1399,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B43">
         <v>2</v>
@@ -1406,15 +1422,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B44">
         <v>2</v>
       </c>
       <c r="C44">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -1429,15 +1445,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B45">
         <v>2</v>
       </c>
       <c r="C45">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -1452,15 +1468,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B46">
         <v>2</v>
       </c>
       <c r="C46">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -1475,15 +1491,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B47">
         <v>2</v>
       </c>
       <c r="C47">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D47">
         <v>1</v>
@@ -1498,15 +1514,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B48">
         <v>2</v>
       </c>
       <c r="C48">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D48">
         <v>1</v>
@@ -1521,15 +1537,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
       <c r="C49">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -1544,15 +1560,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B50">
         <v>2</v>
       </c>
       <c r="C50">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -1567,15 +1583,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B51">
         <v>2</v>
       </c>
       <c r="C51">
-        <v>0.2105</v>
+        <v>0.21049999999999999</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -1590,15 +1606,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B52">
         <v>4</v>
       </c>
       <c r="C52">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -1613,15 +1629,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B53">
         <v>4</v>
       </c>
       <c r="C53">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -1636,15 +1652,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B54">
         <v>4</v>
       </c>
       <c r="C54">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -1659,15 +1675,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B55">
         <v>4</v>
       </c>
       <c r="C55">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -1682,15 +1698,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B56">
         <v>4</v>
       </c>
       <c r="C56">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -1705,15 +1721,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B57">
         <v>4</v>
       </c>
       <c r="C57">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -1728,15 +1744,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B58">
         <v>4</v>
       </c>
       <c r="C58">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -1751,15 +1767,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B59">
         <v>4</v>
       </c>
       <c r="C59">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -1774,15 +1790,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B60">
         <v>4</v>
       </c>
       <c r="C60">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -1797,15 +1813,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B61">
         <v>4</v>
       </c>
       <c r="C61">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -1820,15 +1836,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B62">
         <v>4</v>
       </c>
       <c r="C62">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -1843,15 +1859,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B63">
         <v>4</v>
       </c>
       <c r="C63">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -1866,15 +1882,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B64">
         <v>4</v>
       </c>
       <c r="C64">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -1889,15 +1905,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B65">
         <v>4</v>
       </c>
       <c r="C65">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -1912,15 +1928,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B66">
         <v>4</v>
       </c>
       <c r="C66">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D66">
         <v>1</v>
@@ -1935,15 +1951,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B67">
         <v>4</v>
       </c>
       <c r="C67">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D67">
         <v>1</v>
@@ -1958,15 +1974,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B68">
         <v>4</v>
       </c>
       <c r="C68">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D68">
         <v>1</v>
@@ -1981,15 +1997,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B69">
         <v>4</v>
       </c>
       <c r="C69">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D69">
         <v>1</v>
@@ -2004,15 +2020,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B70">
         <v>4</v>
       </c>
       <c r="C70">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D70">
         <v>1</v>
@@ -2027,15 +2043,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B71">
         <v>4</v>
       </c>
       <c r="C71">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D71">
         <v>1</v>
@@ -2050,15 +2066,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B72">
         <v>4</v>
       </c>
       <c r="C72">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D72">
         <v>1</v>
@@ -2073,15 +2089,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B73">
         <v>4</v>
       </c>
       <c r="C73">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D73">
         <v>1</v>
@@ -2096,15 +2112,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B74">
         <v>4</v>
       </c>
       <c r="C74">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D74">
         <v>1</v>
@@ -2119,15 +2135,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B75">
         <v>4</v>
       </c>
       <c r="C75">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D75">
         <v>1</v>
@@ -2142,15 +2158,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B76">
         <v>4</v>
       </c>
       <c r="C76">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D76">
         <v>1</v>
@@ -2165,15 +2181,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B77">
         <v>4</v>
       </c>
       <c r="C77">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D77">
         <v>1</v>
@@ -2188,15 +2204,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B78">
         <v>4</v>
       </c>
       <c r="C78">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D78">
         <v>1</v>
@@ -2211,15 +2227,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B79">
         <v>4</v>
       </c>
       <c r="C79">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D79">
         <v>1</v>
@@ -2234,15 +2250,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B80">
         <v>4</v>
       </c>
       <c r="C80">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D80">
         <v>1</v>
@@ -2257,15 +2273,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B81">
         <v>4</v>
       </c>
       <c r="C81">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D81">
         <v>1</v>
@@ -2280,15 +2296,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B82">
         <v>4</v>
       </c>
       <c r="C82">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D82">
         <v>1</v>
@@ -2303,15 +2319,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B83">
         <v>4</v>
       </c>
       <c r="C83">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D83">
         <v>1</v>
@@ -2326,15 +2342,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B84">
         <v>4</v>
       </c>
       <c r="C84">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D84">
         <v>1</v>
@@ -2349,15 +2365,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B85">
         <v>4</v>
       </c>
       <c r="C85">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D85">
         <v>1</v>
@@ -2372,15 +2388,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B86">
         <v>4</v>
       </c>
       <c r="C86">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D86">
         <v>1</v>
@@ -2395,15 +2411,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B87">
         <v>4</v>
       </c>
       <c r="C87">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D87">
         <v>1</v>
@@ -2418,15 +2434,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B88">
         <v>4</v>
       </c>
       <c r="C88">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D88">
         <v>1</v>
@@ -2441,15 +2457,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B89">
         <v>4</v>
       </c>
       <c r="C89">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D89">
         <v>1</v>
@@ -2464,15 +2480,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B90">
         <v>4</v>
       </c>
       <c r="C90">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D90">
         <v>1</v>
@@ -2487,15 +2503,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B91">
         <v>4</v>
       </c>
       <c r="C91">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D91">
         <v>1</v>
@@ -2510,15 +2526,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B92">
         <v>4</v>
       </c>
       <c r="C92">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D92">
         <v>1</v>
@@ -2533,15 +2549,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B93">
         <v>4</v>
       </c>
       <c r="C93">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D93">
         <v>1</v>
@@ -2556,15 +2572,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B94">
         <v>4</v>
       </c>
       <c r="C94">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D94">
         <v>1</v>
@@ -2579,15 +2595,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B95">
         <v>4</v>
       </c>
       <c r="C95">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D95">
         <v>1</v>
@@ -2602,15 +2618,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B96">
         <v>4</v>
       </c>
       <c r="C96">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D96">
         <v>1</v>
@@ -2625,15 +2641,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B97">
         <v>4</v>
       </c>
       <c r="C97">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D97">
         <v>1</v>
@@ -2648,15 +2664,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B98">
         <v>4</v>
       </c>
       <c r="C98">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D98">
         <v>1</v>
@@ -2671,15 +2687,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B99">
         <v>4</v>
       </c>
       <c r="C99">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D99">
         <v>1</v>
@@ -2694,15 +2710,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B100">
         <v>4</v>
       </c>
       <c r="C100">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D100">
         <v>1</v>
@@ -2717,15 +2733,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B101">
         <v>4</v>
       </c>
       <c r="C101">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D101">
         <v>1</v>
@@ -2740,7 +2756,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>0.125</v>
       </c>
@@ -2748,7 +2764,7 @@
         <v>8</v>
       </c>
       <c r="C102">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D102">
         <v>1</v>
@@ -2763,7 +2779,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>0.125</v>
       </c>
@@ -2771,7 +2787,7 @@
         <v>8</v>
       </c>
       <c r="C103">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D103">
         <v>1</v>
@@ -2786,7 +2802,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>0.125</v>
       </c>
@@ -2794,7 +2810,7 @@
         <v>8</v>
       </c>
       <c r="C104">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D104">
         <v>1</v>
@@ -2809,7 +2825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>0.125</v>
       </c>
@@ -2817,7 +2833,7 @@
         <v>8</v>
       </c>
       <c r="C105">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D105">
         <v>1</v>
@@ -2832,7 +2848,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>0.125</v>
       </c>
@@ -2840,7 +2856,7 @@
         <v>8</v>
       </c>
       <c r="C106">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D106">
         <v>1</v>
@@ -2855,7 +2871,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>0.125</v>
       </c>
@@ -2863,7 +2879,7 @@
         <v>8</v>
       </c>
       <c r="C107">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D107">
         <v>1</v>
@@ -2878,7 +2894,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>0.125</v>
       </c>
@@ -2886,7 +2902,7 @@
         <v>8</v>
       </c>
       <c r="C108">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D108">
         <v>1</v>
@@ -2901,7 +2917,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>0.125</v>
       </c>
@@ -2909,7 +2925,7 @@
         <v>8</v>
       </c>
       <c r="C109">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D109">
         <v>1</v>
@@ -2924,7 +2940,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:7">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>0.125</v>
       </c>
@@ -2932,7 +2948,7 @@
         <v>8</v>
       </c>
       <c r="C110">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D110">
         <v>1</v>
@@ -2947,7 +2963,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="111" spans="1:7">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>0.125</v>
       </c>
@@ -2955,7 +2971,7 @@
         <v>8</v>
       </c>
       <c r="C111">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D111">
         <v>1</v>
@@ -2970,7 +2986,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="112" spans="1:7">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>0.125</v>
       </c>
@@ -2978,7 +2994,7 @@
         <v>8</v>
       </c>
       <c r="C112">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D112">
         <v>1</v>
@@ -2993,7 +3009,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:7">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>0.125</v>
       </c>
@@ -3001,7 +3017,7 @@
         <v>8</v>
       </c>
       <c r="C113">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D113">
         <v>1</v>
@@ -3016,7 +3032,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="114" spans="1:7">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>0.125</v>
       </c>
@@ -3024,7 +3040,7 @@
         <v>8</v>
       </c>
       <c r="C114">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D114">
         <v>1</v>
@@ -3039,7 +3055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:7">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>0.125</v>
       </c>
@@ -3047,7 +3063,7 @@
         <v>8</v>
       </c>
       <c r="C115">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D115">
         <v>1</v>
@@ -3062,7 +3078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="116" spans="1:7">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>0.125</v>
       </c>
@@ -3070,7 +3086,7 @@
         <v>8</v>
       </c>
       <c r="C116">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D116">
         <v>1</v>
@@ -3085,7 +3101,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="117" spans="1:7">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>0.125</v>
       </c>
@@ -3093,7 +3109,7 @@
         <v>8</v>
       </c>
       <c r="C117">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D117">
         <v>1</v>
@@ -3108,7 +3124,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="118" spans="1:7">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>0.125</v>
       </c>
@@ -3116,7 +3132,7 @@
         <v>8</v>
       </c>
       <c r="C118">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D118">
         <v>1</v>
@@ -3131,7 +3147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:7">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>0.125</v>
       </c>
@@ -3139,7 +3155,7 @@
         <v>8</v>
       </c>
       <c r="C119">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D119">
         <v>1</v>
@@ -3154,7 +3170,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="120" spans="1:7">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>0.125</v>
       </c>
@@ -3162,7 +3178,7 @@
         <v>8</v>
       </c>
       <c r="C120">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D120">
         <v>1</v>
@@ -3177,7 +3193,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="121" spans="1:7">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>0.125</v>
       </c>
@@ -3185,7 +3201,7 @@
         <v>8</v>
       </c>
       <c r="C121">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D121">
         <v>1</v>
@@ -3200,7 +3216,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="122" spans="1:7">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>0.125</v>
       </c>
@@ -3208,7 +3224,7 @@
         <v>8</v>
       </c>
       <c r="C122">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D122">
         <v>1</v>
@@ -3223,7 +3239,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="123" spans="1:7">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>0.125</v>
       </c>
@@ -3231,7 +3247,7 @@
         <v>8</v>
       </c>
       <c r="C123">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D123">
         <v>1</v>
@@ -3246,7 +3262,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="1:7">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>0.125</v>
       </c>
@@ -3254,7 +3270,7 @@
         <v>8</v>
       </c>
       <c r="C124">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D124">
         <v>1</v>
@@ -3269,7 +3285,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:7">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>0.125</v>
       </c>
@@ -3277,7 +3293,7 @@
         <v>8</v>
       </c>
       <c r="C125">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D125">
         <v>1</v>
@@ -3292,7 +3308,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:7">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>0.125</v>
       </c>
@@ -3300,7 +3316,7 @@
         <v>8</v>
       </c>
       <c r="C126">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D126">
         <v>1</v>
@@ -3315,7 +3331,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="127" spans="1:7">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>0.125</v>
       </c>
@@ -3323,7 +3339,7 @@
         <v>8</v>
       </c>
       <c r="C127">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D127">
         <v>1</v>
@@ -3338,7 +3354,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="128" spans="1:7">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>0.125</v>
       </c>
@@ -3346,7 +3362,7 @@
         <v>8</v>
       </c>
       <c r="C128">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D128">
         <v>1</v>
@@ -3361,7 +3377,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="1:7">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>0.125</v>
       </c>
@@ -3369,7 +3385,7 @@
         <v>8</v>
       </c>
       <c r="C129">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D129">
         <v>1</v>
@@ -3384,7 +3400,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="130" spans="1:7">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>0.125</v>
       </c>
@@ -3392,7 +3408,7 @@
         <v>8</v>
       </c>
       <c r="C130">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D130">
         <v>1</v>
@@ -3407,7 +3423,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="131" spans="1:7">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>0.125</v>
       </c>
@@ -3415,7 +3431,7 @@
         <v>8</v>
       </c>
       <c r="C131">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D131">
         <v>1</v>
@@ -3430,7 +3446,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>0.125</v>
       </c>
@@ -3438,7 +3454,7 @@
         <v>8</v>
       </c>
       <c r="C132">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D132">
         <v>1</v>
@@ -3453,7 +3469,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="133" spans="1:7">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>0.125</v>
       </c>
@@ -3461,7 +3477,7 @@
         <v>8</v>
       </c>
       <c r="C133">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D133">
         <v>1</v>
@@ -3476,7 +3492,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:7">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>0.125</v>
       </c>
@@ -3484,7 +3500,7 @@
         <v>8</v>
       </c>
       <c r="C134">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="D134">
         <v>1</v>
@@ -3499,7 +3515,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>0.125</v>
       </c>
@@ -3507,7 +3523,7 @@
         <v>8</v>
       </c>
       <c r="C135">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D135">
         <v>1</v>
@@ -3522,7 +3538,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="136" spans="1:7">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>0.125</v>
       </c>
@@ -3530,7 +3546,7 @@
         <v>8</v>
       </c>
       <c r="C136">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D136">
         <v>1</v>
@@ -3545,7 +3561,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="137" spans="1:7">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>0.125</v>
       </c>
@@ -3553,7 +3569,7 @@
         <v>8</v>
       </c>
       <c r="C137">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D137">
         <v>1</v>
@@ -3568,7 +3584,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:7">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>0.125</v>
       </c>
@@ -3576,7 +3592,7 @@
         <v>8</v>
       </c>
       <c r="C138">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D138">
         <v>1</v>
@@ -3591,7 +3607,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="139" spans="1:7">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>0.125</v>
       </c>
@@ -3599,7 +3615,7 @@
         <v>8</v>
       </c>
       <c r="C139">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D139">
         <v>1</v>
@@ -3614,7 +3630,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>0.125</v>
       </c>
@@ -3622,7 +3638,7 @@
         <v>8</v>
       </c>
       <c r="C140">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D140">
         <v>1</v>
@@ -3637,7 +3653,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="141" spans="1:7">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>0.125</v>
       </c>
@@ -3645,7 +3661,7 @@
         <v>8</v>
       </c>
       <c r="C141">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D141">
         <v>1</v>
@@ -3660,7 +3676,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="142" spans="1:7">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>0.125</v>
       </c>
@@ -3668,7 +3684,7 @@
         <v>8</v>
       </c>
       <c r="C142">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D142">
         <v>1</v>
@@ -3683,7 +3699,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="143" spans="1:7">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>0.125</v>
       </c>
@@ -3691,7 +3707,7 @@
         <v>8</v>
       </c>
       <c r="C143">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D143">
         <v>1</v>
@@ -3706,7 +3722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="144" spans="1:7">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>0.125</v>
       </c>
@@ -3714,7 +3730,7 @@
         <v>8</v>
       </c>
       <c r="C144">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D144">
         <v>1</v>
@@ -3729,7 +3745,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="1:7">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>0.125</v>
       </c>
@@ -3737,7 +3753,7 @@
         <v>8</v>
       </c>
       <c r="C145">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D145">
         <v>1</v>
@@ -3752,7 +3768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:7">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>0.125</v>
       </c>
@@ -3760,7 +3776,7 @@
         <v>8</v>
       </c>
       <c r="C146">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D146">
         <v>1</v>
@@ -3775,7 +3791,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:7">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>0.125</v>
       </c>
@@ -3783,7 +3799,7 @@
         <v>8</v>
       </c>
       <c r="C147">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D147">
         <v>1</v>
@@ -3798,7 +3814,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="148" spans="1:7">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>0.125</v>
       </c>
@@ -3806,7 +3822,7 @@
         <v>8</v>
       </c>
       <c r="C148">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D148">
         <v>1</v>
@@ -3821,7 +3837,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="149" spans="1:7">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>0.125</v>
       </c>
@@ -3829,7 +3845,7 @@
         <v>8</v>
       </c>
       <c r="C149">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D149">
         <v>1</v>
@@ -3844,7 +3860,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="150" spans="1:7">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>0.125</v>
       </c>
@@ -3852,7 +3868,7 @@
         <v>8</v>
       </c>
       <c r="C150">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D150">
         <v>1</v>
@@ -3867,7 +3883,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="151" spans="1:7">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>0.125</v>
       </c>
@@ -3875,7 +3891,7 @@
         <v>8</v>
       </c>
       <c r="C151">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D151">
         <v>1</v>
@@ -3890,7 +3906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="152" spans="1:7">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>0.25</v>
       </c>
@@ -3898,7 +3914,7 @@
         <v>16</v>
       </c>
       <c r="C152">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D152">
         <v>1</v>
@@ -3913,7 +3929,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="153" spans="1:7">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>0.25</v>
       </c>
@@ -3921,7 +3937,7 @@
         <v>16</v>
       </c>
       <c r="C153">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D153">
         <v>1</v>
@@ -3936,7 +3952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>0.25</v>
       </c>
@@ -3944,7 +3960,7 @@
         <v>16</v>
       </c>
       <c r="C154">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D154">
         <v>1</v>
@@ -3959,7 +3975,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="155" spans="1:7">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>0.25</v>
       </c>
@@ -3967,7 +3983,7 @@
         <v>16</v>
       </c>
       <c r="C155">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D155">
         <v>1</v>
@@ -3982,7 +3998,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="156" spans="1:7">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>0.25</v>
       </c>
@@ -3990,7 +4006,7 @@
         <v>16</v>
       </c>
       <c r="C156">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D156">
         <v>1</v>
@@ -4005,7 +4021,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="1:7">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>0.25</v>
       </c>
@@ -4013,7 +4029,7 @@
         <v>16</v>
       </c>
       <c r="C157">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D157">
         <v>1</v>
@@ -4028,7 +4044,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="158" spans="1:7">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>0.25</v>
       </c>
@@ -4036,7 +4052,7 @@
         <v>16</v>
       </c>
       <c r="C158">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D158">
         <v>1</v>
@@ -4051,7 +4067,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="159" spans="1:7">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>0.25</v>
       </c>
@@ -4059,7 +4075,7 @@
         <v>16</v>
       </c>
       <c r="C159">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D159">
         <v>1</v>
@@ -4074,7 +4090,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="160" spans="1:7">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>0.25</v>
       </c>
@@ -4082,7 +4098,7 @@
         <v>16</v>
       </c>
       <c r="C160">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D160">
         <v>1</v>
@@ -4097,7 +4113,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="161" spans="1:7">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>0.25</v>
       </c>
@@ -4105,7 +4121,7 @@
         <v>16</v>
       </c>
       <c r="C161">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D161">
         <v>1</v>
@@ -4120,7 +4136,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:7">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>0.25</v>
       </c>
@@ -4128,7 +4144,7 @@
         <v>16</v>
       </c>
       <c r="C162">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D162">
         <v>1</v>
@@ -4143,7 +4159,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="163" spans="1:7">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>0.25</v>
       </c>
@@ -4151,7 +4167,7 @@
         <v>16</v>
       </c>
       <c r="C163">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D163">
         <v>1</v>
@@ -4166,7 +4182,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="164" spans="1:7">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>0.25</v>
       </c>
@@ -4174,7 +4190,7 @@
         <v>16</v>
       </c>
       <c r="C164">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D164">
         <v>1</v>
@@ -4189,7 +4205,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:7">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>0.25</v>
       </c>
@@ -4197,7 +4213,7 @@
         <v>16</v>
       </c>
       <c r="C165">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D165">
         <v>1</v>
@@ -4212,7 +4228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="166" spans="1:7">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>0.25</v>
       </c>
@@ -4220,7 +4236,7 @@
         <v>16</v>
       </c>
       <c r="C166">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D166">
         <v>1</v>
@@ -4235,7 +4251,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="167" spans="1:7">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>0.25</v>
       </c>
@@ -4243,7 +4259,7 @@
         <v>16</v>
       </c>
       <c r="C167">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D167">
         <v>1</v>
@@ -4258,7 +4274,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="168" spans="1:7">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>0.25</v>
       </c>
@@ -4266,7 +4282,7 @@
         <v>16</v>
       </c>
       <c r="C168">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D168">
         <v>1</v>
@@ -4281,7 +4297,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="1:7">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>0.25</v>
       </c>
@@ -4289,7 +4305,7 @@
         <v>16</v>
       </c>
       <c r="C169">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D169">
         <v>1</v>
@@ -4304,7 +4320,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="170" spans="1:7">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>0.25</v>
       </c>
@@ -4312,7 +4328,7 @@
         <v>16</v>
       </c>
       <c r="C170">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D170">
         <v>1</v>
@@ -4327,7 +4343,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="171" spans="1:7">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>0.25</v>
       </c>
@@ -4335,7 +4351,7 @@
         <v>16</v>
       </c>
       <c r="C171">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D171">
         <v>1</v>
@@ -4350,7 +4366,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="172" spans="1:7">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>0.25</v>
       </c>
@@ -4358,7 +4374,7 @@
         <v>16</v>
       </c>
       <c r="C172">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D172">
         <v>1</v>
@@ -4373,7 +4389,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="173" spans="1:7">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>0.25</v>
       </c>
@@ -4381,7 +4397,7 @@
         <v>16</v>
       </c>
       <c r="C173">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D173">
         <v>1</v>
@@ -4396,7 +4412,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="174" spans="1:7">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>0.25</v>
       </c>
@@ -4404,7 +4420,7 @@
         <v>16</v>
       </c>
       <c r="C174">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D174">
         <v>1</v>
@@ -4419,7 +4435,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="175" spans="1:7">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>0.25</v>
       </c>
@@ -4427,7 +4443,7 @@
         <v>16</v>
       </c>
       <c r="C175">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D175">
         <v>1</v>
@@ -4442,7 +4458,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="176" spans="1:7">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>0.25</v>
       </c>
@@ -4450,7 +4466,7 @@
         <v>16</v>
       </c>
       <c r="C176">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D176">
         <v>1</v>
@@ -4465,7 +4481,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:7">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>0.25</v>
       </c>
@@ -4473,7 +4489,7 @@
         <v>16</v>
       </c>
       <c r="C177">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D177">
         <v>1</v>
@@ -4488,7 +4504,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="178" spans="1:7">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>0.25</v>
       </c>
@@ -4496,7 +4512,7 @@
         <v>16</v>
       </c>
       <c r="C178">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D178">
         <v>1</v>
@@ -4511,7 +4527,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="179" spans="1:7">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>0.25</v>
       </c>
@@ -4519,7 +4535,7 @@
         <v>16</v>
       </c>
       <c r="C179">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D179">
         <v>1</v>
@@ -4534,7 +4550,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="180" spans="1:7">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>0.25</v>
       </c>
@@ -4542,7 +4558,7 @@
         <v>16</v>
       </c>
       <c r="C180">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D180">
         <v>1</v>
@@ -4557,7 +4573,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="181" spans="1:7">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>0.25</v>
       </c>
@@ -4565,7 +4581,7 @@
         <v>16</v>
       </c>
       <c r="C181">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D181">
         <v>1</v>
@@ -4580,7 +4596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="182" spans="1:7">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>0.25</v>
       </c>
@@ -4588,7 +4604,7 @@
         <v>16</v>
       </c>
       <c r="C182">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D182">
         <v>1</v>
@@ -4603,7 +4619,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="183" spans="1:7">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>0.25</v>
       </c>
@@ -4611,7 +4627,7 @@
         <v>16</v>
       </c>
       <c r="C183">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D183">
         <v>1</v>
@@ -4626,7 +4642,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="184" spans="1:7">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>0.25</v>
       </c>
@@ -4634,7 +4650,7 @@
         <v>16</v>
       </c>
       <c r="C184">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D184">
         <v>1</v>
@@ -4649,7 +4665,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="185" spans="1:7">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>0.25</v>
       </c>
@@ -4657,7 +4673,7 @@
         <v>16</v>
       </c>
       <c r="C185">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D185">
         <v>1</v>
@@ -4672,7 +4688,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="186" spans="1:7">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>0.25</v>
       </c>
@@ -4680,7 +4696,7 @@
         <v>16</v>
       </c>
       <c r="C186">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D186">
         <v>1</v>
@@ -4695,7 +4711,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="187" spans="1:7">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>0.25</v>
       </c>
@@ -4703,7 +4719,7 @@
         <v>16</v>
       </c>
       <c r="C187">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D187">
         <v>1</v>
@@ -4718,7 +4734,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="188" spans="1:7">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>0.25</v>
       </c>
@@ -4726,7 +4742,7 @@
         <v>16</v>
       </c>
       <c r="C188">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D188">
         <v>1</v>
@@ -4741,7 +4757,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="189" spans="1:7">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>0.25</v>
       </c>
@@ -4749,7 +4765,7 @@
         <v>16</v>
       </c>
       <c r="C189">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D189">
         <v>1</v>
@@ -4764,7 +4780,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="190" spans="1:7">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>0.25</v>
       </c>
@@ -4772,7 +4788,7 @@
         <v>16</v>
       </c>
       <c r="C190">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D190">
         <v>1</v>
@@ -4787,7 +4803,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="191" spans="1:7">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>0.25</v>
       </c>
@@ -4795,7 +4811,7 @@
         <v>16</v>
       </c>
       <c r="C191">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D191">
         <v>1</v>
@@ -4810,7 +4826,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="192" spans="1:7">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>0.25</v>
       </c>
@@ -4818,7 +4834,7 @@
         <v>16</v>
       </c>
       <c r="C192">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D192">
         <v>1</v>
@@ -4833,7 +4849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="193" spans="1:7">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>0.25</v>
       </c>
@@ -4841,7 +4857,7 @@
         <v>16</v>
       </c>
       <c r="C193">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D193">
         <v>1</v>
@@ -4856,7 +4872,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="194" spans="1:7">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>0.25</v>
       </c>
@@ -4864,7 +4880,7 @@
         <v>16</v>
       </c>
       <c r="C194">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D194">
         <v>1</v>
@@ -4879,7 +4895,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="195" spans="1:7">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>0.25</v>
       </c>
@@ -4887,7 +4903,7 @@
         <v>16</v>
       </c>
       <c r="C195">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D195">
         <v>1</v>
@@ -4902,7 +4918,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="196" spans="1:7">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>0.25</v>
       </c>
@@ -4910,7 +4926,7 @@
         <v>16</v>
       </c>
       <c r="C196">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D196">
         <v>1</v>
@@ -4925,7 +4941,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="197" spans="1:7">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>0.25</v>
       </c>
@@ -4933,7 +4949,7 @@
         <v>16</v>
       </c>
       <c r="C197">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D197">
         <v>1</v>
@@ -4948,7 +4964,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="198" spans="1:7">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>0.25</v>
       </c>
@@ -4956,7 +4972,7 @@
         <v>16</v>
       </c>
       <c r="C198">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D198">
         <v>1</v>
@@ -4971,7 +4987,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="199" spans="1:7">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>0.25</v>
       </c>
@@ -4979,7 +4995,7 @@
         <v>16</v>
       </c>
       <c r="C199">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D199">
         <v>1</v>
@@ -4994,7 +5010,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="200" spans="1:7">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>0.25</v>
       </c>
@@ -5002,7 +5018,7 @@
         <v>16</v>
       </c>
       <c r="C200">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="D200">
         <v>1</v>
@@ -5017,7 +5033,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:7">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>0.25</v>
       </c>
@@ -5025,7 +5041,7 @@
         <v>16</v>
       </c>
       <c r="C201">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D201">
         <v>1</v>
@@ -5040,7 +5056,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:7">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>0.5</v>
       </c>
@@ -5048,7 +5064,7 @@
         <v>32</v>
       </c>
       <c r="C202">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D202">
         <v>1</v>
@@ -5063,7 +5079,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="203" spans="1:7">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>0.5</v>
       </c>
@@ -5071,7 +5087,7 @@
         <v>32</v>
       </c>
       <c r="C203">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D203">
         <v>1</v>
@@ -5086,7 +5102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="204" spans="1:7">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>0.5</v>
       </c>
@@ -5094,7 +5110,7 @@
         <v>32</v>
       </c>
       <c r="C204">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D204">
         <v>1</v>
@@ -5109,7 +5125,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="205" spans="1:7">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>0.5</v>
       </c>
@@ -5117,7 +5133,7 @@
         <v>32</v>
       </c>
       <c r="C205">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D205">
         <v>1</v>
@@ -5132,7 +5148,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="206" spans="1:7">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>0.5</v>
       </c>
@@ -5140,7 +5156,7 @@
         <v>32</v>
       </c>
       <c r="C206">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D206">
         <v>1</v>
@@ -5155,7 +5171,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="207" spans="1:7">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>0.5</v>
       </c>
@@ -5163,7 +5179,7 @@
         <v>32</v>
       </c>
       <c r="C207">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D207">
         <v>1</v>
@@ -5178,7 +5194,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="208" spans="1:7">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>0.5</v>
       </c>
@@ -5186,7 +5202,7 @@
         <v>32</v>
       </c>
       <c r="C208">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D208">
         <v>1</v>
@@ -5201,7 +5217,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="209" spans="1:7">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>0.5</v>
       </c>
@@ -5209,7 +5225,7 @@
         <v>32</v>
       </c>
       <c r="C209">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D209">
         <v>1</v>
@@ -5224,7 +5240,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="210" spans="1:7">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>0.5</v>
       </c>
@@ -5232,7 +5248,7 @@
         <v>32</v>
       </c>
       <c r="C210">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D210">
         <v>1</v>
@@ -5247,7 +5263,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="211" spans="1:7">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>0.5</v>
       </c>
@@ -5255,7 +5271,7 @@
         <v>32</v>
       </c>
       <c r="C211">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D211">
         <v>1</v>
@@ -5270,7 +5286,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="212" spans="1:7">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>0.5</v>
       </c>
@@ -5278,7 +5294,7 @@
         <v>32</v>
       </c>
       <c r="C212">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D212">
         <v>1</v>
@@ -5293,7 +5309,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="213" spans="1:7">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>0.5</v>
       </c>
@@ -5301,7 +5317,7 @@
         <v>32</v>
       </c>
       <c r="C213">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D213">
         <v>1</v>
@@ -5316,7 +5332,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="214" spans="1:7">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>0.5</v>
       </c>
@@ -5324,7 +5340,7 @@
         <v>32</v>
       </c>
       <c r="C214">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D214">
         <v>1</v>
@@ -5339,7 +5355,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="215" spans="1:7">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>0.5</v>
       </c>
@@ -5347,7 +5363,7 @@
         <v>32</v>
       </c>
       <c r="C215">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D215">
         <v>1</v>
@@ -5362,7 +5378,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="216" spans="1:7">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>0.5</v>
       </c>
@@ -5370,7 +5386,7 @@
         <v>32</v>
       </c>
       <c r="C216">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D216">
         <v>1</v>
@@ -5385,7 +5401,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="217" spans="1:7">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>0.5</v>
       </c>
@@ -5393,7 +5409,7 @@
         <v>32</v>
       </c>
       <c r="C217">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D217">
         <v>1</v>
@@ -5408,7 +5424,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="218" spans="1:7">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>0.5</v>
       </c>
@@ -5416,7 +5432,7 @@
         <v>32</v>
       </c>
       <c r="C218">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D218">
         <v>1</v>
@@ -5431,7 +5447,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="219" spans="1:7">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>0.5</v>
       </c>
@@ -5439,7 +5455,7 @@
         <v>32</v>
       </c>
       <c r="C219">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D219">
         <v>1</v>
@@ -5454,7 +5470,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="220" spans="1:7">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>0.5</v>
       </c>
@@ -5462,7 +5478,7 @@
         <v>32</v>
       </c>
       <c r="C220">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D220">
         <v>1</v>
@@ -5477,7 +5493,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="221" spans="1:7">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>0.5</v>
       </c>
@@ -5485,7 +5501,7 @@
         <v>32</v>
       </c>
       <c r="C221">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D221">
         <v>1</v>
@@ -5500,7 +5516,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="222" spans="1:7">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>0.5</v>
       </c>
@@ -5508,7 +5524,7 @@
         <v>32</v>
       </c>
       <c r="C222">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D222">
         <v>1</v>
@@ -5523,7 +5539,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="223" spans="1:7">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>0.5</v>
       </c>
@@ -5531,7 +5547,7 @@
         <v>32</v>
       </c>
       <c r="C223">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D223">
         <v>1</v>
@@ -5546,7 +5562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="224" spans="1:7">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>0.5</v>
       </c>
@@ -5554,7 +5570,7 @@
         <v>32</v>
       </c>
       <c r="C224">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D224">
         <v>1</v>
@@ -5569,7 +5585,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="225" spans="1:7">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>0.5</v>
       </c>
@@ -5577,7 +5593,7 @@
         <v>32</v>
       </c>
       <c r="C225">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D225">
         <v>1</v>
@@ -5592,7 +5608,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="226" spans="1:7">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>0.5</v>
       </c>
@@ -5600,7 +5616,7 @@
         <v>32</v>
       </c>
       <c r="C226">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D226">
         <v>1</v>
@@ -5615,7 +5631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="227" spans="1:7">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>0.5</v>
       </c>
@@ -5623,7 +5639,7 @@
         <v>32</v>
       </c>
       <c r="C227">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D227">
         <v>1</v>
@@ -5638,7 +5654,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="228" spans="1:7">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>0.5</v>
       </c>
@@ -5646,7 +5662,7 @@
         <v>32</v>
       </c>
       <c r="C228">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D228">
         <v>1</v>
@@ -5661,7 +5677,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="229" spans="1:7">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>0.5</v>
       </c>
@@ -5669,7 +5685,7 @@
         <v>32</v>
       </c>
       <c r="C229">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D229">
         <v>1</v>
@@ -5684,7 +5700,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="230" spans="1:7">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>0.5</v>
       </c>
@@ -5692,7 +5708,7 @@
         <v>32</v>
       </c>
       <c r="C230">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D230">
         <v>1</v>
@@ -5707,7 +5723,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="231" spans="1:7">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>0.5</v>
       </c>
@@ -5715,7 +5731,7 @@
         <v>32</v>
       </c>
       <c r="C231">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D231">
         <v>1</v>
@@ -5730,7 +5746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="232" spans="1:7">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>0.5</v>
       </c>
@@ -5738,7 +5754,7 @@
         <v>32</v>
       </c>
       <c r="C232">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D232">
         <v>1</v>
@@ -5753,7 +5769,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="233" spans="1:7">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>0.5</v>
       </c>
@@ -5761,7 +5777,7 @@
         <v>32</v>
       </c>
       <c r="C233">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D233">
         <v>1</v>
@@ -5776,7 +5792,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="234" spans="1:7">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>0.5</v>
       </c>
@@ -5784,7 +5800,7 @@
         <v>32</v>
       </c>
       <c r="C234">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D234">
         <v>1</v>
@@ -5799,7 +5815,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="235" spans="1:7">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>0.5</v>
       </c>
@@ -5807,7 +5823,7 @@
         <v>32</v>
       </c>
       <c r="C235">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D235">
         <v>1</v>
@@ -5822,7 +5838,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="236" spans="1:7">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>0.5</v>
       </c>
@@ -5830,7 +5846,7 @@
         <v>32</v>
       </c>
       <c r="C236">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D236">
         <v>1</v>
@@ -5845,7 +5861,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="237" spans="1:7">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>0.5</v>
       </c>
@@ -5853,7 +5869,7 @@
         <v>32</v>
       </c>
       <c r="C237">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D237">
         <v>1</v>
@@ -5868,7 +5884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="238" spans="1:7">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>0.5</v>
       </c>
@@ -5876,7 +5892,7 @@
         <v>32</v>
       </c>
       <c r="C238">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D238">
         <v>1</v>
@@ -5891,7 +5907,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="239" spans="1:7">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>0.5</v>
       </c>
@@ -5899,7 +5915,7 @@
         <v>32</v>
       </c>
       <c r="C239">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D239">
         <v>1</v>
@@ -5914,7 +5930,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="240" spans="1:7">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>0.5</v>
       </c>
@@ -5922,7 +5938,7 @@
         <v>32</v>
       </c>
       <c r="C240">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D240">
         <v>1</v>
@@ -5937,7 +5953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="241" spans="1:7">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>0.5</v>
       </c>
@@ -5945,7 +5961,7 @@
         <v>32</v>
       </c>
       <c r="C241">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D241">
         <v>1</v>
@@ -5960,7 +5976,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="242" spans="1:7">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>0.5</v>
       </c>
@@ -5968,7 +5984,7 @@
         <v>32</v>
       </c>
       <c r="C242">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D242">
         <v>1</v>
@@ -5983,7 +5999,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="243" spans="1:7">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>0.5</v>
       </c>
@@ -5991,7 +6007,7 @@
         <v>32</v>
       </c>
       <c r="C243">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D243">
         <v>1</v>
@@ -6006,7 +6022,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="244" spans="1:7">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>0.5</v>
       </c>
@@ -6014,7 +6030,7 @@
         <v>32</v>
       </c>
       <c r="C244">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D244">
         <v>1</v>
@@ -6029,7 +6045,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:7">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>0.5</v>
       </c>
@@ -6037,7 +6053,7 @@
         <v>32</v>
       </c>
       <c r="C245">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D245">
         <v>1</v>
@@ -6052,7 +6068,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="246" spans="1:7">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>0.5</v>
       </c>
@@ -6060,7 +6076,7 @@
         <v>32</v>
       </c>
       <c r="C246">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D246">
         <v>1</v>
@@ -6075,7 +6091,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="247" spans="1:7">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>0.5</v>
       </c>
@@ -6083,7 +6099,7 @@
         <v>32</v>
       </c>
       <c r="C247">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D247">
         <v>1</v>
@@ -6098,7 +6114,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="248" spans="1:7">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>0.5</v>
       </c>
@@ -6106,7 +6122,7 @@
         <v>32</v>
       </c>
       <c r="C248">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D248">
         <v>1</v>
@@ -6121,7 +6137,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="249" spans="1:7">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>0.5</v>
       </c>
@@ -6129,7 +6145,7 @@
         <v>32</v>
       </c>
       <c r="C249">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D249">
         <v>1</v>
@@ -6144,7 +6160,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="250" spans="1:7">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>0.5</v>
       </c>
@@ -6152,7 +6168,7 @@
         <v>32</v>
       </c>
       <c r="C250">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D250">
         <v>1</v>
@@ -6167,7 +6183,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="251" spans="1:7">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>0.5</v>
       </c>
@@ -6175,7 +6191,7 @@
         <v>32</v>
       </c>
       <c r="C251">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D251">
         <v>1</v>
@@ -6196,11 +6212,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="71.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6235,9 +6263,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>0.03125</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -6249,7 +6277,7 @@
         <v>0.1053</v>
       </c>
       <c r="E2">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -6270,21 +6298,21 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>0.0625</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
       <c r="C3">
-        <v>0.273708</v>
+        <v>0.27370800000000001</v>
       </c>
       <c r="D3">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="E3">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -6305,7 +6333,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0.125</v>
       </c>
@@ -6313,13 +6341,13 @@
         <v>8</v>
       </c>
       <c r="C4">
-        <v>0.284238</v>
+        <v>0.28423799999999999</v>
       </c>
       <c r="D4">
-        <v>0.2368</v>
+        <v>0.23680000000000001</v>
       </c>
       <c r="E4">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -6340,7 +6368,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>0.25</v>
       </c>
@@ -6348,13 +6376,13 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>0.286344</v>
+        <v>0.28634399999999999</v>
       </c>
       <c r="D5">
-        <v>0.2632</v>
+        <v>0.26319999999999999</v>
       </c>
       <c r="E5">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -6375,7 +6403,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>0.5</v>
       </c>
@@ -6383,13 +6411,13 @@
         <v>32</v>
       </c>
       <c r="C6">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="D6">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="E6">
-        <v>0.2895</v>
+        <v>0.28949999999999998</v>
       </c>
       <c r="F6">
         <v>1</v>

</xml_diff>